<commit_message>
Stage 8 fixes: E-001
</commit_message>
<xml_diff>
--- a/output/archive/WestravelleData/Stability/CVL/WA-2020-313/Results/Approved/CVL_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
+++ b/output/archive/WestravelleData/Stability/CVL/WA-2020-313/Results/Approved/CVL_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
@@ -173,7 +173,7 @@
   <commentList>
     <comment ref="D4" authorId="0" shapeId="0">
       <text>
-        <t>Impact assessment agreed. No change to the stability conclusion.</t>
+        <t>Read the DN-02 sequence attachment for control results and acceptance disposition. No sequence-level result is reproduced here.</t>
       </text>
     </comment>
   </commentList>
@@ -611,7 +611,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Stability of tablet lot 3 under ICH long-term and accelerated conditions, with the HPLC assay and related-substances method qualified before the first pull. Pulls at 0, 3, 6, 9 and 12 months. The six-month interim review was completed on 31 May 2021.</t>
+          <t>Stability of tablet lot 3 under ICH long-term, intermediate and accelerated conditions. Long-term and intermediate pulls at 0, 1, 3, 6, 9 and 12 months; accelerated pulls at 0, 1, 3 and 6 months. Interim review: 31 May 2021.</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1292,7 +1292,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Validated before the first stability pull under the assay and related-substances validation protocol. Acceptance criteria as written in the protocol.</t>
+          <t>Method validation establishes method performance; it is not sequence-level system suitability. Validation criteria and results are tabulated below.</t>
         </is>
       </c>
     </row>
@@ -1433,6 +1433,27 @@
       <c r="C12" s="2" t="inlineStr">
         <is>
           <t>≤0.05</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Sequence-level source records</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>For each condition/timepoint on Pulls, consult the corresponding WA/2020/313 sequence sheet linked from batch card WST-20-009708. That record carries the sequence identifier, control injections, method-specific control criteria, observed results and acceptance signature. These details are not transcribed here; this validation table must not be used to infer sequence acceptance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Replacement-column sequence: consult the sequence attachment to DN-02 and the column-change entry in the same batch card. Control criteria and acceptance disposition belong to that sequence record; no replacement-column control result is asserted here.</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1542,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Chromatography column replaced between the interim review and the nine-month pull. System suitability repeated before the sequence was run.</t>
+          <t>Column replacement noted between interim review and nine-month pull. DN-02 and its sequence attachment are the source for replacement-column sequence identifier, controls, criteria and disposition; method validation does not establish repeat suitability.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">

</xml_diff>